<commit_message>
Rebuild China/India workbooks with new Wave 1A rule
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01WLyHMjDC3dbaNBgTG82etS
</commit_message>
<xml_diff>
--- a/research/brics_universities/output/BRICS_universities_China.xlsx
+++ b/research/brics_universities/output/BRICS_universities_China.xlsx
@@ -482,7 +482,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Дата формирования: 2026-10-02</t>
+          <t>Дата формирования: 2026-10-04</t>
         </is>
       </c>
     </row>
@@ -580,7 +580,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Волна 1A: есть запущенные КА и индекс ≥ 60. Волна 1B: новые члены БРИКС+ и ключевые точки для наземных станций (индекс ≥ 40).</t>
+          <t>Волна 1A: у вуза есть собственные запущенные КА. Волна 1B: новые члены БРИКС+ и ключевые точки для наземных станций (индекс ≥ 40).</t>
         </is>
       </c>
     </row>
@@ -1042,7 +1042,7 @@
       </c>
       <c r="AH2" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI2" s="4" t="inlineStr">
@@ -1242,7 +1242,7 @@
       </c>
       <c r="AH3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI3" s="4" t="inlineStr">
@@ -1445,7 +1445,7 @@
       </c>
       <c r="AH4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI4" s="4" t="inlineStr">
@@ -1644,7 +1644,7 @@
       </c>
       <c r="AH5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI5" s="4" t="inlineStr">
@@ -1847,7 +1847,7 @@
       </c>
       <c r="AH6" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI6" s="4" t="inlineStr">
@@ -2038,7 +2038,7 @@
       </c>
       <c r="AH7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI7" s="4" t="inlineStr">
@@ -2214,7 +2214,7 @@
       </c>
       <c r="AH8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI8" s="4" t="inlineStr">
@@ -2401,7 +2401,7 @@
       </c>
       <c r="AH9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI9" s="4" t="inlineStr">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="AH10" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI10" s="4" t="inlineStr"/>
@@ -2767,7 +2767,7 @@
       </c>
       <c r="AH11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI11" s="4" t="inlineStr">
@@ -2955,7 +2955,7 @@
       </c>
       <c r="AH12" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI12" s="4" t="inlineStr">
@@ -3138,7 +3138,7 @@
       </c>
       <c r="AH13" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI13" s="4" t="inlineStr"/>
@@ -3327,7 +3327,7 @@
       </c>
       <c r="AH14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI14" s="4" t="inlineStr">
@@ -3513,7 +3513,7 @@
       </c>
       <c r="AH15" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI15" s="4" t="inlineStr">
@@ -3723,7 +3723,7 @@
       </c>
       <c r="AH16" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI16" s="4" t="inlineStr">
@@ -3906,7 +3906,7 @@
       </c>
       <c r="AH17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI17" s="4" t="inlineStr">
@@ -4094,7 +4094,7 @@
       </c>
       <c r="AH18" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI18" s="4" t="inlineStr">
@@ -4290,7 +4290,7 @@
       </c>
       <c r="AH19" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI19" s="4" t="inlineStr">
@@ -4485,7 +4485,7 @@
       </c>
       <c r="AH20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI20" s="4" t="inlineStr">
@@ -4658,7 +4658,7 @@
       </c>
       <c r="AH21" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI21" s="4" t="inlineStr">
@@ -4837,7 +4837,7 @@
       </c>
       <c r="AH22" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI22" s="4" t="inlineStr"/>
@@ -5009,7 +5009,7 @@
       </c>
       <c r="AH23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI23" s="4" t="inlineStr">
@@ -5177,7 +5177,7 @@
       </c>
       <c r="AH24" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI24" s="4" t="inlineStr">
@@ -5366,7 +5366,7 @@
       </c>
       <c r="AH25" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI25" s="4" t="inlineStr">
@@ -5546,7 +5546,7 @@
       </c>
       <c r="AH26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI26" s="4" t="inlineStr"/>
@@ -5717,7 +5717,7 @@
       </c>
       <c r="AH27" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI27" s="4" t="inlineStr">
@@ -5888,7 +5888,7 @@
       </c>
       <c r="AH28" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI28" s="4" t="inlineStr">
@@ -6071,7 +6071,7 @@
       </c>
       <c r="AH29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI29" s="4" t="inlineStr">
@@ -6252,7 +6252,7 @@
       </c>
       <c r="AH30" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI30" s="4" t="inlineStr">
@@ -6424,7 +6424,7 @@
       </c>
       <c r="AH31" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI31" s="4" t="inlineStr"/>
@@ -6600,7 +6600,7 @@
       </c>
       <c r="AH32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI32" s="4" t="inlineStr">
@@ -6772,7 +6772,7 @@
       </c>
       <c r="AH33" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI33" s="4" t="inlineStr"/>
@@ -6949,7 +6949,7 @@
       </c>
       <c r="AH34" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI34" s="4" t="inlineStr">
@@ -7103,7 +7103,7 @@
       </c>
       <c r="AH35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI35" s="4" t="inlineStr">
@@ -7279,7 +7279,7 @@
       </c>
       <c r="AH36" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI36" s="4" t="inlineStr">
@@ -7443,7 +7443,7 @@
       </c>
       <c r="AH37" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI37" s="4" t="inlineStr">
@@ -7862,7 +7862,7 @@
       </c>
       <c r="AH2" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI2" s="4" t="inlineStr">
@@ -8062,7 +8062,7 @@
       </c>
       <c r="AH3" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI3" s="4" t="inlineStr">
@@ -8265,7 +8265,7 @@
       </c>
       <c r="AH4" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI4" s="4" t="inlineStr">
@@ -8464,7 +8464,7 @@
       </c>
       <c r="AH5" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI5" s="4" t="inlineStr">
@@ -8667,7 +8667,7 @@
       </c>
       <c r="AH6" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI6" s="4" t="inlineStr">
@@ -8858,7 +8858,7 @@
       </c>
       <c r="AH7" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI7" s="4" t="inlineStr">
@@ -9034,7 +9034,7 @@
       </c>
       <c r="AH8" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI8" s="4" t="inlineStr">
@@ -9221,7 +9221,7 @@
       </c>
       <c r="AH9" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI9" s="4" t="inlineStr">
@@ -9403,7 +9403,7 @@
       </c>
       <c r="AH10" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI10" s="4" t="inlineStr"/>
@@ -9587,7 +9587,7 @@
       </c>
       <c r="AH11" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI11" s="4" t="inlineStr">
@@ -9775,7 +9775,7 @@
       </c>
       <c r="AH12" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI12" s="4" t="inlineStr">
@@ -9958,7 +9958,7 @@
       </c>
       <c r="AH13" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI13" s="4" t="inlineStr"/>
@@ -10147,7 +10147,7 @@
       </c>
       <c r="AH14" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI14" s="4" t="inlineStr">
@@ -10333,7 +10333,7 @@
       </c>
       <c r="AH15" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI15" s="4" t="inlineStr">
@@ -10543,7 +10543,7 @@
       </c>
       <c r="AH16" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI16" s="4" t="inlineStr">
@@ -10726,7 +10726,7 @@
       </c>
       <c r="AH17" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI17" s="4" t="inlineStr">
@@ -10914,7 +10914,7 @@
       </c>
       <c r="AH18" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI18" s="4" t="inlineStr">
@@ -11110,7 +11110,7 @@
       </c>
       <c r="AH19" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI19" s="4" t="inlineStr">
@@ -11305,7 +11305,7 @@
       </c>
       <c r="AH20" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI20" s="4" t="inlineStr">
@@ -11478,7 +11478,7 @@
       </c>
       <c r="AH21" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI21" s="4" t="inlineStr">
@@ -11657,7 +11657,7 @@
       </c>
       <c r="AH22" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI22" s="4" t="inlineStr"/>
@@ -11829,7 +11829,7 @@
       </c>
       <c r="AH23" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI23" s="4" t="inlineStr">
@@ -11997,7 +11997,7 @@
       </c>
       <c r="AH24" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI24" s="4" t="inlineStr">
@@ -12186,7 +12186,7 @@
       </c>
       <c r="AH25" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI25" s="4" t="inlineStr">
@@ -12366,7 +12366,7 @@
       </c>
       <c r="AH26" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI26" s="4" t="inlineStr"/>
@@ -12537,7 +12537,7 @@
       </c>
       <c r="AH27" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI27" s="4" t="inlineStr">
@@ -12708,7 +12708,7 @@
       </c>
       <c r="AH28" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI28" s="4" t="inlineStr">
@@ -12891,7 +12891,7 @@
       </c>
       <c r="AH29" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI29" s="4" t="inlineStr">
@@ -13072,7 +13072,7 @@
       </c>
       <c r="AH30" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI30" s="4" t="inlineStr">
@@ -13244,7 +13244,7 @@
       </c>
       <c r="AH31" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI31" s="4" t="inlineStr"/>
@@ -13420,7 +13420,7 @@
       </c>
       <c r="AH32" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI32" s="4" t="inlineStr">
@@ -13592,7 +13592,7 @@
       </c>
       <c r="AH33" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI33" s="4" t="inlineStr"/>
@@ -13769,7 +13769,7 @@
       </c>
       <c r="AH34" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI34" s="4" t="inlineStr">
@@ -13923,7 +13923,7 @@
       </c>
       <c r="AH35" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI35" s="4" t="inlineStr">
@@ -14099,7 +14099,7 @@
       </c>
       <c r="AH36" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI36" s="4" t="inlineStr">
@@ -14263,7 +14263,7 @@
       </c>
       <c r="AH37" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI37" s="4" t="inlineStr">
@@ -14442,7 +14442,7 @@
       </c>
       <c r="AH38" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI38" s="4" t="inlineStr">
@@ -14616,7 +14616,7 @@
       </c>
       <c r="AH39" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI39" s="4" t="inlineStr">
@@ -14778,7 +14778,7 @@
       </c>
       <c r="AH40" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI40" s="4" t="inlineStr">
@@ -14945,7 +14945,7 @@
       </c>
       <c r="AH41" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI41" s="4" t="inlineStr">
@@ -15119,7 +15119,7 @@
       </c>
       <c r="AH42" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI42" s="4" t="inlineStr">
@@ -15296,7 +15296,7 @@
       </c>
       <c r="AH43" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI43" s="4" t="inlineStr">
@@ -15471,7 +15471,7 @@
       </c>
       <c r="AH44" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI44" s="4" t="inlineStr">
@@ -15652,7 +15652,7 @@
       </c>
       <c r="AH45" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI45" s="4" t="inlineStr">
@@ -15823,7 +15823,7 @@
       </c>
       <c r="AH46" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI46" s="4" t="inlineStr">
@@ -15995,7 +15995,7 @@
       </c>
       <c r="AH47" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI47" s="4" t="inlineStr">
@@ -16167,7 +16167,7 @@
       </c>
       <c r="AH48" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI48" s="4" t="inlineStr">
@@ -16333,7 +16333,7 @@
       </c>
       <c r="AH49" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI49" s="4" t="inlineStr">
@@ -16504,7 +16504,7 @@
       </c>
       <c r="AH50" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI50" s="4" t="inlineStr">
@@ -16678,7 +16678,7 @@
       </c>
       <c r="AH51" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI51" s="4" t="inlineStr">
@@ -16849,7 +16849,7 @@
       </c>
       <c r="AH52" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI52" s="4" t="inlineStr">
@@ -17020,7 +17020,7 @@
       </c>
       <c r="AH53" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI53" s="4" t="inlineStr"/>
@@ -17189,7 +17189,7 @@
       </c>
       <c r="AH54" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI54" s="4" t="inlineStr">
@@ -17363,7 +17363,7 @@
       </c>
       <c r="AH55" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI55" s="4" t="inlineStr">
@@ -17534,7 +17534,7 @@
       </c>
       <c r="AH56" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI56" s="4" t="inlineStr">
@@ -17700,7 +17700,7 @@
       </c>
       <c r="AH57" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI57" s="4" t="inlineStr">
@@ -17868,7 +17868,7 @@
       </c>
       <c r="AH58" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI58" s="4" t="inlineStr">
@@ -18037,7 +18037,7 @@
       </c>
       <c r="AH59" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI59" s="4" t="inlineStr">
@@ -18210,7 +18210,7 @@
       </c>
       <c r="AH60" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI60" s="4" t="inlineStr">
@@ -18379,7 +18379,7 @@
       </c>
       <c r="AH61" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI61" s="4" t="inlineStr">
@@ -18525,7 +18525,7 @@
       </c>
       <c r="AH62" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI62" s="4" t="inlineStr">
@@ -18691,7 +18691,7 @@
       </c>
       <c r="AH63" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI63" s="4" t="inlineStr">
@@ -18851,7 +18851,7 @@
       </c>
       <c r="AH64" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI64" s="4" t="inlineStr">
@@ -19019,7 +19019,7 @@
       </c>
       <c r="AH65" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI65" s="4" t="inlineStr">
@@ -19185,7 +19185,7 @@
       </c>
       <c r="AH66" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI66" s="4" t="inlineStr"/>
@@ -19340,7 +19340,7 @@
       </c>
       <c r="AH67" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI67" s="4" t="inlineStr">
@@ -19502,7 +19502,7 @@
       </c>
       <c r="AH68" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI68" s="4" t="inlineStr">
@@ -19636,7 +19636,7 @@
       </c>
       <c r="AD69" s="4" t="inlineStr">
         <is>
-          <t>нет</t>
+          <t>да</t>
         </is>
       </c>
       <c r="AE69" s="4" t="inlineStr">
@@ -19664,7 +19664,7 @@
       </c>
       <c r="AH69" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI69" s="4" t="inlineStr">
@@ -19825,7 +19825,7 @@
       </c>
       <c r="AH70" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI70" s="4" t="inlineStr">
@@ -19986,7 +19986,7 @@
       </c>
       <c r="AH71" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI71" s="4" t="inlineStr"/>
@@ -20145,7 +20145,7 @@
       </c>
       <c r="AH72" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI72" s="4" t="inlineStr">
@@ -20303,7 +20303,7 @@
       </c>
       <c r="AH73" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI73" s="4" t="inlineStr">
@@ -20471,7 +20471,7 @@
       </c>
       <c r="AH74" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI74" s="4" t="inlineStr">
@@ -20631,7 +20631,7 @@
       </c>
       <c r="AH75" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI75" s="4" t="inlineStr">
@@ -20789,7 +20789,7 @@
       </c>
       <c r="AH76" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI76" s="4" t="inlineStr">
@@ -20946,7 +20946,7 @@
       </c>
       <c r="AH77" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI77" s="4" t="inlineStr">
@@ -21102,7 +21102,7 @@
       </c>
       <c r="AH78" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI78" s="4" t="inlineStr">
@@ -21263,7 +21263,7 @@
       </c>
       <c r="AH79" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI79" s="4" t="inlineStr">
@@ -21409,7 +21409,7 @@
       </c>
       <c r="AH80" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI80" s="4" t="inlineStr">
@@ -21576,7 +21576,7 @@
       </c>
       <c r="AH81" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI81" s="4" t="inlineStr">
@@ -21742,7 +21742,7 @@
       </c>
       <c r="AH82" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI82" s="4" t="inlineStr">
@@ -21881,7 +21881,7 @@
       </c>
       <c r="AH83" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI83" s="4" t="inlineStr">
@@ -22039,7 +22039,7 @@
       </c>
       <c r="AH84" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI84" s="4" t="inlineStr">
@@ -22197,7 +22197,7 @@
       </c>
       <c r="AH85" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI85" s="4" t="inlineStr">
@@ -22367,7 +22367,7 @@
       </c>
       <c r="AH86" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI86" s="4" t="inlineStr">
@@ -22524,7 +22524,7 @@
       </c>
       <c r="AH87" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI87" s="4" t="inlineStr">
@@ -22660,7 +22660,7 @@
       </c>
       <c r="AH88" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI88" s="4" t="inlineStr">
@@ -22792,7 +22792,7 @@
       </c>
       <c r="AH89" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI89" s="4" t="inlineStr">
@@ -22948,7 +22948,7 @@
       </c>
       <c r="AH90" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI90" s="4" t="inlineStr">
@@ -23108,7 +23108,7 @@
       </c>
       <c r="AH91" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI91" s="4" t="inlineStr">
@@ -23247,7 +23247,7 @@
       </c>
       <c r="AH92" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI92" s="4" t="inlineStr">
@@ -23406,7 +23406,7 @@
       </c>
       <c r="AH93" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI93" s="4" t="inlineStr">
@@ -23531,7 +23531,7 @@
       </c>
       <c r="AH94" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI94" s="4" t="inlineStr">
@@ -23687,7 +23687,7 @@
       </c>
       <c r="AH95" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI95" s="4" t="inlineStr">
@@ -23827,7 +23827,7 @@
       </c>
       <c r="AH96" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI96" s="4" t="inlineStr">
@@ -23989,7 +23989,7 @@
       </c>
       <c r="AH97" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI97" s="4" t="inlineStr">
@@ -24146,7 +24146,7 @@
       </c>
       <c r="AH98" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI98" s="4" t="inlineStr">
@@ -24298,7 +24298,7 @@
       </c>
       <c r="AH99" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI99" s="4" t="inlineStr">
@@ -24459,7 +24459,7 @@
       </c>
       <c r="AH100" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI100" s="4" t="inlineStr">
@@ -24612,7 +24612,7 @@
       </c>
       <c r="AH101" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI101" s="4" t="inlineStr">
@@ -24769,7 +24769,7 @@
       </c>
       <c r="AH102" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI102" s="4" t="inlineStr">
@@ -24905,7 +24905,7 @@
       </c>
       <c r="AH103" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI103" s="4" t="inlineStr">
@@ -25057,7 +25057,7 @@
       </c>
       <c r="AH104" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI104" s="4" t="inlineStr">
@@ -25185,7 +25185,7 @@
       </c>
       <c r="AH105" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI105" s="4" t="inlineStr">
@@ -25341,7 +25341,7 @@
       </c>
       <c r="AH106" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI106" s="4" t="inlineStr">
@@ -25497,7 +25497,7 @@
       </c>
       <c r="AH107" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI107" s="4" t="inlineStr">
@@ -25656,7 +25656,7 @@
       </c>
       <c r="AH108" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI108" s="4" t="inlineStr">
@@ -25811,7 +25811,7 @@
       </c>
       <c r="AH109" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI109" s="4" t="inlineStr">
@@ -25963,7 +25963,7 @@
       </c>
       <c r="AH110" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI110" s="4" t="inlineStr">
@@ -26120,7 +26120,7 @@
       </c>
       <c r="AH111" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI111" s="4" t="inlineStr">
@@ -26278,7 +26278,7 @@
       </c>
       <c r="AH112" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI112" s="4" t="inlineStr">
@@ -26406,7 +26406,7 @@
       </c>
       <c r="AH113" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI113" s="4" t="inlineStr"/>
@@ -26557,7 +26557,7 @@
       </c>
       <c r="AH114" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI114" s="4" t="inlineStr">
@@ -26713,7 +26713,7 @@
       </c>
       <c r="AH115" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI115" s="4" t="inlineStr">
@@ -26848,7 +26848,7 @@
       </c>
       <c r="AH116" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI116" s="4" t="inlineStr">
@@ -27008,7 +27008,7 @@
       </c>
       <c r="AH117" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI117" s="4" t="inlineStr">
@@ -27160,7 +27160,7 @@
       </c>
       <c r="AH118" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI118" s="4" t="inlineStr">
@@ -27298,7 +27298,7 @@
       </c>
       <c r="AH119" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI119" s="4" t="inlineStr">
@@ -27455,7 +27455,7 @@
       </c>
       <c r="AH120" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI120" s="4" t="inlineStr">
@@ -27615,7 +27615,7 @@
       </c>
       <c r="AH121" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI121" s="4" t="inlineStr">
@@ -27768,7 +27768,7 @@
       </c>
       <c r="AH122" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI122" s="4" t="inlineStr">
@@ -27923,7 +27923,7 @@
       </c>
       <c r="AH123" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI123" s="4" t="inlineStr">
@@ -28077,7 +28077,7 @@
       </c>
       <c r="AH124" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI124" s="4" t="inlineStr">
@@ -28234,7 +28234,7 @@
       </c>
       <c r="AH125" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI125" s="4" t="inlineStr">
@@ -28375,7 +28375,7 @@
       </c>
       <c r="AH126" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI126" s="4" t="inlineStr">
@@ -28532,7 +28532,7 @@
       </c>
       <c r="AH127" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI127" s="4" t="inlineStr">
@@ -28664,7 +28664,7 @@
       </c>
       <c r="AH128" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI128" s="4" t="inlineStr">
@@ -28819,7 +28819,7 @@
       </c>
       <c r="AH129" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI129" s="4" t="inlineStr">
@@ -28977,7 +28977,7 @@
       </c>
       <c r="AH130" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI130" s="4" t="inlineStr">
@@ -29137,7 +29137,7 @@
       </c>
       <c r="AH131" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI131" s="4" t="inlineStr">
@@ -29271,7 +29271,7 @@
       </c>
       <c r="AH132" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI132" s="4" t="inlineStr">
@@ -29397,7 +29397,7 @@
       </c>
       <c r="AH133" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI133" s="4" t="inlineStr"/>
@@ -29544,7 +29544,7 @@
       </c>
       <c r="AH134" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI134" s="4" t="inlineStr">
@@ -29699,7 +29699,7 @@
       </c>
       <c r="AH135" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI135" s="4" t="inlineStr">
@@ -29824,7 +29824,7 @@
       </c>
       <c r="AH136" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI136" s="4" t="inlineStr">
@@ -29973,7 +29973,7 @@
       </c>
       <c r="AH137" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI137" s="4" t="inlineStr">
@@ -30099,7 +30099,7 @@
       </c>
       <c r="AH138" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI138" s="4" t="inlineStr">
@@ -30223,7 +30223,7 @@
       </c>
       <c r="AH139" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI139" s="4" t="inlineStr">
@@ -30382,7 +30382,7 @@
       </c>
       <c r="AH140" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI140" s="4" t="inlineStr">
@@ -30534,7 +30534,7 @@
       </c>
       <c r="AH141" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI141" s="4" t="inlineStr">
@@ -30683,7 +30683,7 @@
       </c>
       <c r="AH142" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI142" s="4" t="inlineStr">
@@ -30835,7 +30835,7 @@
       </c>
       <c r="AH143" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI143" s="4" t="inlineStr">
@@ -30983,7 +30983,7 @@
       </c>
       <c r="AH144" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI144" s="4" t="inlineStr">
@@ -31115,7 +31115,7 @@
       </c>
       <c r="AH145" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI145" s="4" t="inlineStr">
@@ -31267,7 +31267,7 @@
       </c>
       <c r="AH146" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI146" s="4" t="inlineStr">
@@ -31420,7 +31420,7 @@
       </c>
       <c r="AH147" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI147" s="4" t="inlineStr">
@@ -31570,7 +31570,7 @@
       </c>
       <c r="AH148" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI148" s="4" t="inlineStr">
@@ -31717,7 +31717,7 @@
       </c>
       <c r="AH149" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI149" s="4" t="inlineStr">
@@ -31867,7 +31867,7 @@
       </c>
       <c r="AH150" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI150" s="4" t="inlineStr">
@@ -32019,7 +32019,7 @@
       </c>
       <c r="AH151" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI151" s="4" t="inlineStr">
@@ -32130,7 +32130,7 @@
       </c>
       <c r="AH152" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI152" s="4" t="inlineStr"/>
@@ -32230,7 +32230,7 @@
       </c>
       <c r="AH153" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI153" s="4" t="inlineStr"/>
@@ -32369,7 +32369,7 @@
       </c>
       <c r="AH154" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI154" s="4" t="inlineStr">
@@ -32516,7 +32516,7 @@
       </c>
       <c r="AH155" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI155" s="4" t="inlineStr"/>
@@ -32664,7 +32664,7 @@
       </c>
       <c r="AH156" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI156" s="4" t="inlineStr">
@@ -32819,7 +32819,7 @@
       </c>
       <c r="AH157" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI157" s="4" t="inlineStr">
@@ -32968,7 +32968,7 @@
       </c>
       <c r="AH158" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI158" s="4" t="inlineStr">
@@ -33118,7 +33118,7 @@
       </c>
       <c r="AH159" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI159" s="4" t="inlineStr">
@@ -33248,7 +33248,7 @@
       </c>
       <c r="AH160" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI160" s="4" t="inlineStr">
@@ -33373,7 +33373,7 @@
       </c>
       <c r="AH161" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI161" s="4" t="inlineStr">
@@ -33508,7 +33508,7 @@
       </c>
       <c r="AH162" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI162" s="4" t="inlineStr">
@@ -33657,7 +33657,7 @@
       </c>
       <c r="AH163" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI163" s="4" t="inlineStr">
@@ -33813,7 +33813,7 @@
       </c>
       <c r="AH164" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI164" s="4" t="inlineStr">
@@ -33935,7 +33935,7 @@
       </c>
       <c r="AH165" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI165" s="4" t="inlineStr">
@@ -34064,7 +34064,7 @@
       </c>
       <c r="AH166" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI166" s="4" t="inlineStr">
@@ -34215,7 +34215,7 @@
       </c>
       <c r="AH167" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI167" s="4" t="inlineStr">
@@ -34319,7 +34319,7 @@
       </c>
       <c r="AH168" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI168" s="4" t="inlineStr"/>
@@ -34469,7 +34469,7 @@
       </c>
       <c r="AH169" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI169" s="4" t="inlineStr">
@@ -34622,7 +34622,7 @@
       </c>
       <c r="AH170" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI170" s="4" t="inlineStr">
@@ -34745,7 +34745,7 @@
       </c>
       <c r="AH171" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI171" s="4" t="inlineStr"/>
@@ -34893,7 +34893,7 @@
       </c>
       <c r="AH172" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI172" s="4" t="inlineStr">
@@ -35044,7 +35044,7 @@
       </c>
       <c r="AH173" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI173" s="4" t="inlineStr">
@@ -35190,7 +35190,7 @@
       </c>
       <c r="AH174" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI174" s="4" t="inlineStr">
@@ -35342,7 +35342,7 @@
       </c>
       <c r="AH175" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI175" s="4" t="inlineStr">
@@ -35488,7 +35488,7 @@
       </c>
       <c r="AH176" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI176" s="4" t="inlineStr">
@@ -35641,7 +35641,7 @@
       </c>
       <c r="AH177" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI177" s="4" t="inlineStr">
@@ -35775,7 +35775,7 @@
       </c>
       <c r="AH178" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI178" s="4" t="inlineStr">
@@ -35923,7 +35923,7 @@
       </c>
       <c r="AH179" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI179" s="4" t="inlineStr">
@@ -36075,7 +36075,7 @@
       </c>
       <c r="AH180" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI180" s="4" t="inlineStr">
@@ -36199,7 +36199,7 @@
       </c>
       <c r="AH181" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI181" s="4" t="inlineStr">
@@ -36327,7 +36327,7 @@
       </c>
       <c r="AH182" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI182" s="4" t="inlineStr">
@@ -36481,7 +36481,7 @@
       </c>
       <c r="AH183" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI183" s="4" t="inlineStr">
@@ -36630,7 +36630,7 @@
       </c>
       <c r="AH184" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI184" s="4" t="inlineStr">
@@ -36784,7 +36784,7 @@
       </c>
       <c r="AH185" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI185" s="4" t="inlineStr">
@@ -36931,7 +36931,7 @@
       </c>
       <c r="AH186" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI186" s="4" t="inlineStr">
@@ -37084,7 +37084,7 @@
       </c>
       <c r="AH187" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI187" s="4" t="inlineStr">
@@ -37221,7 +37221,7 @@
       </c>
       <c r="AH188" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI188" s="4" t="inlineStr">
@@ -37370,7 +37370,7 @@
       </c>
       <c r="AH189" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI189" s="4" t="inlineStr">
@@ -37484,7 +37484,7 @@
       </c>
       <c r="AH190" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI190" s="4" t="inlineStr"/>
@@ -37627,7 +37627,7 @@
       </c>
       <c r="AH191" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI191" s="4" t="inlineStr">
@@ -37782,7 +37782,7 @@
       </c>
       <c r="AH192" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI192" s="4" t="inlineStr">
@@ -37931,7 +37931,7 @@
       </c>
       <c r="AH193" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI193" s="4" t="inlineStr">
@@ -38079,7 +38079,7 @@
       </c>
       <c r="AH194" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI194" s="4" t="inlineStr">
@@ -38227,7 +38227,7 @@
       </c>
       <c r="AH195" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI195" s="4" t="inlineStr">
@@ -38379,7 +38379,7 @@
       </c>
       <c r="AH196" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI196" s="4" t="inlineStr">
@@ -38526,7 +38526,7 @@
       </c>
       <c r="AH197" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI197" s="4" t="inlineStr">
@@ -38657,7 +38657,7 @@
       </c>
       <c r="AH198" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI198" s="4" t="inlineStr">
@@ -38806,7 +38806,7 @@
       </c>
       <c r="AH199" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI199" s="4" t="inlineStr">
@@ -38954,7 +38954,7 @@
       </c>
       <c r="AH200" s="4" t="inlineStr">
         <is>
-          <t>2026-10-02</t>
+          <t>2026-10-04</t>
         </is>
       </c>
       <c r="AI200" s="4" t="inlineStr">

</xml_diff>